<commit_message>
Sponsor cards: bring back real business logos (finsavy.jpg, chandni-yadav.jpg) in the middle badge via new LogoURL column, move the small Font Awesome icon to sit next to the sponsor's name instead; document how to add a headshot (AvatarURL) in the admin panel description
</commit_message>
<xml_diff>
--- a/data/sponsors.xlsx
+++ b/data/sponsors.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -434,18 +434,19 @@
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,60 +492,65 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>LogoURL</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>BusinessName</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Tagline</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>SocialLabel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>SocialURL</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>CTAText</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>CTALink</t>
         </is>
@@ -587,60 +593,65 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>assets/images/partners/finsavy.jpg</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Finsavvys</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Finances for the Future.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Financial strategies and solutions for all age groups — helping families and individuals plan smart and build lasting wealth.</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Life Insurance, 401K / IRA Rollovers, Retirement Planning, College Savings, Wealth Management, Estate Planning, Tax Efficiency, Long-Term Care</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>finsavvys.com</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>(507) 230-3434</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>teamfinsavvys@gmail.com</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>@finsavvys</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>https://www.instagram.com/finsavvys</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Visit Finsavvys</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>https://finsavvys.com</t>
         </is>
@@ -683,60 +694,65 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>assets/images/partners/chandni-yadav.jpg</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>Chandni Yadav Realty</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Integrity · Knowledgeable · Trustworthy · Committed</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Real Estate · KW Elite</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Helping you build generational wealth through real estate, with personalized guidance for buyers and sellers across Massachusetts and Rhode Island.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Home Buying, Home Selling, Residential Realty, Keller Williams Elite</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>chandniyadav.kw.com</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>(401) 834-9616</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Chandnirealty@gmail.com</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Chandniyadavrealty</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Chandniyadavrealty</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Contact Chandni</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>https://chandniyadav.kw.com</t>
         </is>

</xml_diff>